<commit_message>
Clean workflow configurations and remove hardcoded API secrets
</commit_message>
<xml_diff>
--- a/files/marketing-content-latest.xlsx
+++ b/files/marketing-content-latest.xlsx
@@ -460,7 +460,7 @@
     </row>
     <row r="2" xml:space="preserve">
       <c r="A2" t="str">
-        <v>2026-06-25T14:01:09.383Z</v>
+        <v>2026-06-30T04:19:52.504Z</v>
       </c>
       <c r="B2" t="str">
         <v>Q2 Product Launch</v>
@@ -487,54 +487,43 @@
         <v>gpt-4o-mini-2024-07-18</v>
       </c>
       <c r="J2" t="str">
-        <v>Revolutionizing Marketing Content Creation with n8n's AI Agents</v>
+        <v>Revolutionizing Content Creation: How n8n's AI Agents Empower Marketing Teams</v>
       </c>
       <c r="K2" t="str">
-        <v>Discover how n8n's AI agents streamline your marketing content creation process, enabling B2B SaaS companies to work smarter, not harder.</v>
+        <v>Discover how n8n's AI content agents streamline your marketing efforts, enabling B2B SaaS companies to automate content creation for blogs, social media, and emails.</v>
       </c>
       <c r="L2" t="str" xml:space="preserve">
-        <v xml:space="preserve"># Revolutionizing Marketing Content Creation with n8n's AI Agents
-In today's fast-paced digital landscape, marketing managers are constantly seeking innovative ways to optimize their workflows and enhance productivity. Enter n8n's AI agents—your new best friend in automating marketing content creation.
-## What are n8n AI Agents?
-n8n AI agents are intelligent automation tools designed to simplify the content generation process. Whether you need blog posts, social media updates, or email campaigns, n8n can seamlessly integrate these tasks into one cohesive workflow. 
-## Why Marketing Managers Love n8n
-1. **Efficiency**: Say goodbye to repetitive tasks. With our AI agents, you can focus on strategy while we handle the content creation.
-2. **Consistency**: Ensure that your brand's voice remains consistent across all platforms with AI-generated content tailored to your needs.
-3. **Scalability**: As your content needs grow, n8n scales with you, making it easy to manage larger volumes of content without sacrificing quality.
-### How It Works
-Using n8n, marketing teams can set up automated workflows that trigger content generation based on specific criteria. For instance, you can create a workflow that generates a blog post every time a new product is launched, or schedule social media updates based on your content calendar.
-## Get Started Today
-Ready to take your marketing efforts to the next level? Start your free trial of n8n and experience the power of AI-driven marketing automation. Transform the way you create content and free up your time for what matters most—growing your business!</v>
+        <v xml:space="preserve"># Revolutionizing Content Creation: How n8n's AI Agents Empower Marketing Teams
+In the fast-paced world of B2B SaaS marketing, efficiency is key. Marketing managers face the constant challenge of producing high-quality content across multiple channels while maintaining consistency and engagement. Enter **n8n** – your ultimate solution for **marketing automation**. Our AI agents are designed to simplify and enhance your content creation process.
+## The Power of n8n AI Content Agents
+With n8n's innovative AI content agents, you can automate the creation of blog posts, social media updates, and email campaigns all within a single workflow. This means less time spent on drafting and editing, and more time focused on strategy and growth.
+### Streamline Your Workflow
+Imagine being able to generate a week's worth of social media posts in just a few clicks. Our AI agents can analyze your brand voice and target audience to create tailored content that resonates with your customers. Plus, the seamless integration with your existing tools means you won't have to disrupt your current processes.
+### Enhance Creativity and Engagement
+By automating repetitive tasks, your team can devote more energy to creative strategies that drive engagement. Our AI agents are not just tools; they are collaborators that help you brainstorm ideas, refine messaging, and ensure your content aligns with your marketing goals.
+## Start Your Free Trial Today!
+Ready to take your content creation to the next level? **Start your free trial** of n8n today and see how our AI agents can transform your marketing efforts!</v>
       </c>
       <c r="M2" t="str">
-        <v>🚀 Exciting news for marketing managers! With n8n's AI agents, you can automate your content creation process—from blogs to social media posts—effortlessly. Say goodbye to repetitive tasks and hello to efficiency! Start your free trial today: https://n8n.io</v>
+        <v>🚀 Excited to announce the launch of our AI content agents at n8n! Marketing managers can now automate the creation of blogs, social media posts, and emails in one streamlined workflow. Discover how n8n can boost your marketing efficiency and creativity. Start your free trial today! #n8n #MarketingAutomation #AIContentAgent #ContentCreation #B2BMarketing</v>
       </c>
       <c r="N2" t="str">
-        <v>#MarketingAutomation #AIContentCreation #n8n #B2B #SaaS</v>
+        <v>#n8n #MarketingAutomation #AIContentAgent #ContentCreation #B2BMarketing</v>
       </c>
       <c r="O2" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. 🚀 Attention marketing managers! Did you know that n8n's AI agents can automate your content creation process? From blogs to social media posts, it's all possible with one workflow! #MarketingAutomation #n8n
-2. ✅ Efficiency is key in today's fast-paced world. With n8n, you can focus on strategy while our AI agents handle the content generation for you! #AIContentCreation
-3. 🔗 Ready to transform your marketing efforts? Start your free trial today and see how n8n can revolutionize your content creation process! https://n8n.io #B2B #SaaS</v>
+        <v xml:space="preserve">1. 🚀 Exciting news! n8n is launching AI content agents to revolutionize your marketing efforts! #n8n #MarketingAutomation
+2. With our AI agents, you can automate blog, social media, and email content creation in one seamless workflow. No more hassle! #AIContentAgent
+3. Imagine having more time for strategy and creativity while your AI agents handle the repetitive tasks. #ContentCreation
+4. Ready to enhance your marketing game? Start your free trial of n8n today! #B2BMarketing</v>
       </c>
       <c r="P2" t="str">
-        <v>Transform Your Marketing Content Creation with n8n! | Meet Your New Marketing Assistant: n8n AI Agents | Streamline Your Content Creation Process Today!</v>
+        <v>Transform Your Marketing with n8n's AI Content Agents! | Automate Your Content Creation Process with n8n | Unlock Efficiency in Your Marketing Workflow</v>
       </c>
       <c r="Q2" t="str">
-        <v>Discover how n8n's AI agents can automate your marketing content creation and boost efficiency.</v>
-      </c>
-      <c r="R2" t="str" xml:space="preserve">
-        <v xml:space="preserve">&lt;h1&gt;Transform Your Marketing Content Creation with n8n!&lt;/h1&gt;
-&lt;p&gt;Dear Marketing Manager,&lt;/p&gt;
-&lt;p&gt;Are you looking to optimize your content creation process? Meet n8n's AI agents—your new ally in marketing automation! Our AI-driven tools help you generate blog posts, social media updates, and email campaigns all in one seamless workflow.&lt;/p&gt;
-&lt;p&gt;With n8n, you can:&lt;/p&gt;
-&lt;ul&gt;
-&lt;li&gt;Boost efficiency by automating repetitive tasks&lt;/li&gt;
-&lt;li&gt;Maintain a consistent brand voice across all platforms&lt;/li&gt;
-&lt;li&gt;Scale your content production effortlessly&lt;/li&gt;
-&lt;/ul&gt;
-&lt;p&gt;Ready to take your marketing efforts to the next level? &lt;a href='https://n8n.io'&gt;Start your free trial today&lt;/a&gt; and experience the future of content creation!&lt;/p&gt;
-&lt;p&gt;Best regards,&lt;br&gt;The n8n Team&lt;/p&gt;</v>
+        <v>Discover how n8n's AI agents can streamline your content creation process!</v>
+      </c>
+      <c r="R2" t="str">
+        <v>&lt;html&gt;&lt;body&gt;&lt;h1&gt;Transform Your Marketing with n8n's AI Content Agents!&lt;/h1&gt;&lt;p&gt;Dear Marketing Manager,&lt;/p&gt;&lt;p&gt;We know that producing high-quality content across various channels is crucial for your success in the B2B SaaS landscape. That's why we're excited to introduce n8n's AI content agents, designed to automate your content creation process.&lt;/p&gt;&lt;p&gt;With n8n, you can effortlessly generate blog posts, social media updates, and email campaigns all in one workflow. This means more time for creative strategies and less time on repetitive tasks.&lt;/p&gt;&lt;p&gt;Ready to see how n8n can transform your marketing efforts? &lt;a href='https://n8n.io' target='_blank'&gt;Start your free trial today!&lt;/a&gt;&lt;/p&gt;&lt;p&gt;Best regards,&lt;br&gt;The n8n Team&lt;/p&gt;&lt;/body&gt;&lt;/html&gt;</v>
       </c>
       <c r="S2" t="str">
         <v/>

</xml_diff>